<commit_message>
Contar o atestado da TAMILES como dia trabalhado na meta de setembro
Atestado abonado conta como dia trabalhado: TAMILES fica com 30 dias e a
meta cheia de R$ 12.000,00 no programa de metas de setembro.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_SETEMBRO_2026_TRANCOSO_pgto_05-10-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_SETEMBRO_2026_TRANCOSO_pgto_05-10-2026.xlsx
@@ -2252,7 +2252,7 @@
         <v>12000</v>
       </c>
       <c r="D16" s="27" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E16" s="25">
         <f>ROUND(C16*IF(D16="",0,D16)/30,2)</f>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="T16" s="34" t="inlineStr">
         <is>
-          <t>Atestado de 02 a 08/09: 23 dias trabalhados. Ajustar se o atestado contar como dia trabalhado.</t>
+          <t>Atestado de 02 a 08/09 abonado: conta como dia trabalhado, meta cheia.</t>
         </is>
       </c>
     </row>

</xml_diff>